<commit_message>
V12 update: PLOS section order, Table 3 fix, ethics statement, reference format, compliance check
</commit_message>
<xml_diff>
--- a/Supplementary_Information/S3_Table_Pipeline_Specification.xlsx
+++ b/Supplementary_Information/S3_Table_Pipeline_Specification.xlsx
@@ -704,7 +704,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>ICH E11 assign: 5 age bands; unknown retained</t>
+          <t>ICH E11 assign: 4 bands + Unknown, retained</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Assigns one of five ICH E11(R1) bands; cases with unresolved age are retained as the Unknown band</t>
+          <t>Assigns one of the four ICH E11(R1) bands; cases with unresolved age are retained in the Unknown category</t>
         </is>
       </c>
     </row>

</xml_diff>